<commit_message>
Add a visual survey builder, and reminders in place of stop checks
The builder is one offline HTML page that edits a spec's JSON: a card per
step, a map of the flow's shape, and a WhatsApp preview. It never talks to
Twilio, and rtt survey check stays the check that counts. `just
survey-builder` opens it; an untouched open-and-save is byte-identical,
which a Node test runs against spec_to_dict.

The spec changes with it:

- Stop words are listened for in the opening and in reply to a reminder,
  set once in settings.stop_words, not per question. STOP is understood
  in every language.
- A question sends a no-reply reminder with the question again, at
  settings.reminder_after (23h30, the last moment WhatsApp allows free
  text). timeout_reminder and timeout_message replace stop_check.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_template.xlsx
+++ b/sample_template.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,8 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,20 +537,25 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>stop_check</t>
+          <t>timeout_message</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>timeout_reminder</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>publish</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>encrypt</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>widgets</t>
         </is>
@@ -587,24 +593,25 @@
       <c r="I2" s="3" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr"/>
       <c r="K2" s="3" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -641,24 +648,25 @@
       <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>7</t>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -691,24 +699,25 @@
       <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr"/>
       <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr"/>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -746,24 +755,25 @@
           <t>error_numeric</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -796,24 +806,25 @@
       <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -850,13 +861,14 @@
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr"/>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -895,13 +907,14 @@
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="3" t="inlineStr"/>
       <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr"/>
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr"/>
-      <c r="O8" s="3" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -940,13 +953,14 @@
       <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr"/>
       <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr"/>
-      <c r="O9" s="3" t="inlineStr">
+      <c r="O9" s="3" t="inlineStr"/>
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -985,13 +999,14 @@
       <c r="J10" s="3" t="inlineStr"/>
       <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr"/>
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr"/>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1030,13 +1045,14 @@
       <c r="J11" s="3" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr"/>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1071,13 +1087,14 @@
       <c r="J12" s="3" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr"/>
       <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr"/>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1320,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1393,22 +1410,34 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>stop_words</t>
+          <t>timeout_nudge</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>stop, quit, unsubscribe, cancel, end</t>
+          <t>Just checking in: here is the question again whenever you have a moment. If you would rather stop, reply STOP and we will not message you again.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>stop_words</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>stop, quit, unsubscribe, cancel, end</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>unsolicited</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Thanks for your message. Nothing further is needed.</t>
         </is>
@@ -1425,7 +1454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1531,34 +1560,58 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>preloads</t>
+          <t>stop_words</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>caseid, name, sent_at</t>
+          <t>opening_and_reminders</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>flow_name:en</t>
+          <t>reminder_after</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>my_survey</t>
+          <t>84600</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>preloads</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>caseid, name, sent_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>flow_name:en</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>my_survey</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>description:en</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>One line saying what this round is for</t>
         </is>
@@ -1575,7 +1628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1844,16 +1897,16 @@
       <c r="A46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>stop_check - default yes, and it should stay yes</t>
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>timeout_reminder - default yes. Send the no-reply reminder.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Routes a mid-survey STOP before the reply is treated as an answer. Twilio's own opt-out handling covers the carrier keywords for SMS; inside a WhatsApp session a STOP is an ordinary message and nothing looks at it unless the flow does. Without this, saying stop stores 'stop' as the answer and the next question goes out anyway.</t>
+          <t xml:space="preserve">  When nobody replies for the settings' reminder_after (23h30 unless you change it), the person gets the reminder and the same question again. Then the usual timeout runs; if there is still nothing, they are marked as not replying.</t>
         </is>
       </c>
     </row>
@@ -1861,21 +1914,38 @@
       <c r="A49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>timeout_message - this question's own reminder text</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A key from the messages sheet. Blank uses timeout_nudge. A reminder goes to somebody who has gone quiet, so say they can reply STOP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
         <is>
           <t>publish - default yes. Whether the answer reaches the warehouse.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>encrypt - default no. Encrypt this field before it is stored.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  For direct identifiers only - a name, a phone number.</t>
         </is>
@@ -2044,7 +2114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2073,7 +2143,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Keys this instrument uses: error_option, error_option_labels, error_numeric, list_button, stop_words, unsolicited</t>
+          <t>Keys this instrument uses: error_option, error_option_labels, error_numeric, list_button, timeout_nudge, stop_words, unsolicited</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2173,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>stop_words - comma-separated. Include the English words even in a non-English instrument: people type STOP whatever language they are answering in.</t>
+          <t>stop_words - comma-separated. STOP is always understood, in every language, and capitals do not matter (stop, Stop, STOP). Where they are listened for is the settings' stop_words: by default the opening (opener, consent, first question) and any reply to a reminder. Mid-survey a person who has had enough simply stops answering.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2183,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>list_button - the up-to-20-character button that opens a list.</t>
+          <t>timeout_nudge - the no-reply reminder, sent with the question again after the settings' reminder_after (23h30 by default, the last moment WhatsApp still allows free text). Tell people they can reply STOP.</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2193,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>unsolicited - sent to somebody who writes to the number without having been launched into the survey. In practice that is mostly people being polite after finishing, and re-sending the opener to them would restart the whole survey.</t>
+          <t>list_button - the up-to-20-character button that opens a list.</t>
         </is>
       </c>
     </row>
@@ -2132,6 +2202,16 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>unsolicited - sent to somebody who writes to the number without having been launched into the survey. In practice that is mostly people being polite after finishing, and re-sending the opener to them would restart the whole survey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>{button} in a nudge is filled in with the list button's text, so a nudge cannot name a button that is not on screen.</t>
         </is>

</xml_diff>